<commit_message>
feat: check field name
</commit_message>
<xml_diff>
--- a/test/res/typedef.xlsx
+++ b/test/res/typedef.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/codetypes/Desktop/Github/xlsx-exporter/test/res/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\bite\Desktop\github\xlsx-gen\test\res\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{203FE284-D992-4D47-A4E1-C7F5D59A5BB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DE56734-ADF3-4189-BE65-30DB198BD8D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="17680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="39870" yWindow="810" windowWidth="34995" windowHeight="18885" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="typedef" sheetId="2" r:id="rId1"/>
     <sheet name="main" sheetId="9" r:id="rId2"/>
+    <sheet name="coin" sheetId="10" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">typedef!$A$2:$F$24</definedName>
@@ -896,8 +897,43 @@
 </comments>
 </file>
 
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Administrator</author>
+  </authors>
+  <commentList>
+    <comment ref="C5" authorId="0" shapeId="0" xr:uid="{5BB4E7C5-1B43-4962-9650-892C918B7A3A}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t>条件：和参数一致，是固定的，详见第一张表</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="60">
   <si>
     <t>id</t>
   </si>
@@ -1062,24 +1098,44 @@
   </si>
   <si>
     <t>MonsterTeam?</t>
+  </si>
+  <si>
+    <t>value_checker?</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>string?</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>x</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>检查器</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>#coin.id</t>
+    <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -1100,13 +1156,13 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -1238,7 +1294,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1299,12 +1355,20 @@
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
     <cellStyle name="常规 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000031000000}"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="2">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFF9900"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1588,16 +1652,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:F29"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15"/>
+  <dimension ref="A1:G29"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="24.1640625" customWidth="1"/>
-    <col min="4" max="5" width="21.1640625" customWidth="1"/>
-    <col min="6" max="6" width="20.33203125" customWidth="1"/>
+    <col min="2" max="2" width="14.875" customWidth="1"/>
+    <col min="3" max="3" width="24.125" customWidth="1"/>
+    <col min="4" max="5" width="21.125" customWidth="1"/>
+    <col min="6" max="7" width="20.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="20" t="s">
         <v>18</v>
       </c>
@@ -1606,8 +1670,9 @@
       <c r="D1" s="21"/>
       <c r="E1" s="21"/>
       <c r="F1" s="21"/>
-    </row>
-    <row r="2" spans="1:6" ht="16">
+      <c r="G1" s="22"/>
+    </row>
+    <row r="2" spans="1:7" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -1626,8 +1691,11 @@
       <c r="F2" s="3" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" ht="16">
+      <c r="G2" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>14</v>
       </c>
@@ -1646,8 +1714,11 @@
       <c r="F3" s="3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" ht="16">
+      <c r="G3" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
@@ -1656,8 +1727,9 @@
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
       <c r="F4" s="3"/>
-    </row>
-    <row r="5" spans="1:6" ht="16">
+      <c r="G4" s="3"/>
+    </row>
+    <row r="5" spans="1:7" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>7</v>
       </c>
@@ -1676,8 +1748,11 @@
       <c r="F5" s="3" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" ht="16">
+      <c r="G5" s="3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>8</v>
       </c>
@@ -1690,8 +1765,11 @@
       <c r="F6" s="3" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" ht="16">
+      <c r="G6" s="3" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>16</v>
       </c>
@@ -1710,8 +1788,9 @@
       <c r="F7" s="5" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" ht="16">
+      <c r="G7" s="5"/>
+    </row>
+    <row r="8" spans="1:7" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>16</v>
       </c>
@@ -1728,8 +1807,9 @@
       <c r="F8" s="5" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" ht="16">
+      <c r="G8" s="5"/>
+    </row>
+    <row r="9" spans="1:7" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>16</v>
       </c>
@@ -1746,8 +1826,9 @@
       <c r="F9" s="5" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" ht="16">
+      <c r="G9" s="5"/>
+    </row>
+    <row r="10" spans="1:7" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>16</v>
       </c>
@@ -1764,8 +1845,9 @@
       <c r="F10" s="5" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" ht="16">
+      <c r="G10" s="5"/>
+    </row>
+    <row r="11" spans="1:7" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>16</v>
       </c>
@@ -1784,8 +1866,9 @@
       <c r="F11" s="5" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" ht="16">
+      <c r="G11" s="5"/>
+    </row>
+    <row r="12" spans="1:7" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>16</v>
       </c>
@@ -1802,8 +1885,9 @@
       <c r="F12" s="5" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" ht="16">
+      <c r="G12" s="5"/>
+    </row>
+    <row r="13" spans="1:7" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>16</v>
       </c>
@@ -1822,8 +1906,9 @@
       <c r="F13" s="5" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" ht="16">
+      <c r="G13" s="5"/>
+    </row>
+    <row r="14" spans="1:7" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>16</v>
       </c>
@@ -1840,8 +1925,11 @@
       <c r="F14" s="5" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" ht="16">
+      <c r="G14" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>16</v>
       </c>
@@ -1858,8 +1946,9 @@
       <c r="F15" s="5" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" ht="16">
+      <c r="G15" s="5"/>
+    </row>
+    <row r="16" spans="1:7" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
         <v>16</v>
       </c>
@@ -1876,8 +1965,9 @@
       <c r="F16" s="5" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" ht="16">
+      <c r="G16" s="5"/>
+    </row>
+    <row r="17" spans="1:7" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
         <v>16</v>
       </c>
@@ -1894,102 +1984,115 @@
         <v>21</v>
       </c>
       <c r="F17" s="5"/>
-    </row>
-    <row r="18" spans="1:6" ht="16">
+      <c r="G17" s="5"/>
+    </row>
+    <row r="18" spans="1:7" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A18" s="1"/>
       <c r="B18" s="5"/>
       <c r="C18" s="5"/>
       <c r="D18" s="5"/>
       <c r="E18" s="5"/>
       <c r="F18" s="5"/>
-    </row>
-    <row r="19" spans="1:6" ht="16">
+      <c r="G18" s="5"/>
+    </row>
+    <row r="19" spans="1:7" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A19" s="1"/>
       <c r="B19" s="5"/>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
       <c r="E19" s="4"/>
       <c r="F19" s="4"/>
-    </row>
-    <row r="20" spans="1:6" ht="16">
+      <c r="G19" s="4"/>
+    </row>
+    <row r="20" spans="1:7" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A20" s="1"/>
       <c r="B20" s="2"/>
       <c r="C20" s="6"/>
       <c r="D20" s="6"/>
       <c r="E20" s="6"/>
       <c r="F20" s="6"/>
-    </row>
-    <row r="21" spans="1:6" ht="16">
+      <c r="G20" s="6"/>
+    </row>
+    <row r="21" spans="1:7" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A21" s="1"/>
       <c r="B21" s="2"/>
       <c r="C21" s="6"/>
       <c r="D21" s="6"/>
       <c r="E21" s="6"/>
       <c r="F21" s="6"/>
-    </row>
-    <row r="22" spans="1:6" ht="16">
+      <c r="G21" s="6"/>
+    </row>
+    <row r="22" spans="1:7" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A22" s="1"/>
       <c r="B22" s="2"/>
       <c r="C22" s="6"/>
       <c r="D22" s="6"/>
       <c r="E22" s="6"/>
       <c r="F22" s="6"/>
-    </row>
-    <row r="23" spans="1:6" ht="16">
+      <c r="G22" s="6"/>
+    </row>
+    <row r="23" spans="1:7" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A23" s="1"/>
       <c r="B23" s="2"/>
       <c r="C23" s="6"/>
       <c r="D23" s="6"/>
       <c r="E23" s="6"/>
       <c r="F23" s="6"/>
-    </row>
-    <row r="24" spans="1:6" ht="16">
+      <c r="G23" s="6"/>
+    </row>
+    <row r="24" spans="1:7" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A24" s="1"/>
       <c r="B24" s="2"/>
       <c r="C24" s="6"/>
       <c r="D24" s="6"/>
       <c r="E24" s="6"/>
       <c r="F24" s="6"/>
-    </row>
-    <row r="25" spans="1:6" ht="16">
+      <c r="G24" s="6"/>
+    </row>
+    <row r="25" spans="1:7" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A25" s="1"/>
       <c r="B25" s="7"/>
       <c r="C25" s="8"/>
       <c r="D25" s="4"/>
       <c r="E25" s="4"/>
       <c r="F25" s="8"/>
-    </row>
-    <row r="26" spans="1:6" ht="16">
+      <c r="G25" s="8"/>
+    </row>
+    <row r="26" spans="1:7" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A26" s="1"/>
       <c r="B26" s="7"/>
       <c r="C26" s="8"/>
       <c r="D26" s="4"/>
       <c r="E26" s="4"/>
       <c r="F26" s="8"/>
-    </row>
-    <row r="27" spans="1:6" ht="16">
+      <c r="G26" s="8"/>
+    </row>
+    <row r="27" spans="1:7" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A27" s="1"/>
       <c r="B27" s="7"/>
       <c r="C27" s="8"/>
       <c r="D27" s="4"/>
       <c r="E27" s="4"/>
       <c r="F27" s="8"/>
-    </row>
-    <row r="28" spans="1:6" ht="16">
+      <c r="G27" s="8"/>
+    </row>
+    <row r="28" spans="1:7" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A28" s="1"/>
       <c r="B28" s="7"/>
       <c r="C28" s="8"/>
       <c r="D28" s="4"/>
       <c r="E28" s="4"/>
       <c r="F28" s="8"/>
-    </row>
-    <row r="29" spans="1:6" ht="16">
+      <c r="G28" s="8"/>
+    </row>
+    <row r="29" spans="1:7" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A29" s="1"/>
       <c r="B29" s="7"/>
       <c r="C29" s="8"/>
       <c r="D29" s="4"/>
       <c r="E29" s="4"/>
       <c r="F29" s="8"/>
+      <c r="G29" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2004,13 +2107,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A814D64C-E2BB-9F48-8DDA-58BFAA61AAAE}">
   <dimension ref="A1:D7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="3" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="41.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="41.375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="12" customFormat="1" ht="16">
+    <row r="1" spans="1:4" s="12" customFormat="1" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
@@ -2024,7 +2127,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" s="12" customFormat="1" ht="16">
+    <row r="2" spans="1:4" s="12" customFormat="1" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A2" s="9" t="s">
         <v>4</v>
       </c>
@@ -2038,7 +2141,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="3" spans="1:4" s="12" customFormat="1" ht="16">
+    <row r="3" spans="1:4" s="12" customFormat="1" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A3" s="9" t="s">
         <v>6</v>
       </c>
@@ -2048,7 +2151,7 @@
       <c r="C3" s="11"/>
       <c r="D3" s="11"/>
     </row>
-    <row r="4" spans="1:4" s="12" customFormat="1" ht="16">
+    <row r="4" spans="1:4" s="12" customFormat="1" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A4" s="9" t="s">
         <v>7</v>
       </c>
@@ -2062,7 +2165,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:4" s="12" customFormat="1" ht="16">
+    <row r="5" spans="1:4" s="12" customFormat="1" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A5" s="9" t="s">
         <v>8</v>
       </c>
@@ -2076,7 +2179,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:4" s="12" customFormat="1" ht="17">
+    <row r="6" spans="1:4" s="12" customFormat="1" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A6" s="15">
         <v>1001</v>
       </c>
@@ -2090,7 +2193,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="7" spans="1:4" s="12" customFormat="1" ht="16">
+    <row r="7" spans="1:4" s="12" customFormat="1" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A7" s="15">
         <v>1002</v>
       </c>
@@ -2105,8 +2208,91 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
   <conditionalFormatting sqref="A1:A7">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B463A41-6A33-4F17-9DC2-DDE655130202}">
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="3" max="3" width="15.875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="16.5" x14ac:dyDescent="0.2">
+      <c r="A1" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="11" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="16.5" x14ac:dyDescent="0.2">
+      <c r="A2" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.2">
+      <c r="A3" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" s="11"/>
+    </row>
+    <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.2">
+      <c r="A4" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="16.5" x14ac:dyDescent="0.2">
+      <c r="A5" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="16.5" x14ac:dyDescent="0.2">
+      <c r="A6" s="15">
+        <v>71001</v>
+      </c>
+      <c r="B6" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="C6" s="17" t="s">
+        <v>41</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
+  <conditionalFormatting sqref="A1:A6">
+    <cfRule type="duplicateValues" dxfId="0" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>

</xml_diff>